<commit_message>
adding results for 1 week
</commit_message>
<xml_diff>
--- a/results/greedy_baseline_comparison.xlsx
+++ b/results/greedy_baseline_comparison.xlsx
@@ -5,17 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mmarathe/Documents/GitHub/CATS-CaliforniaTestSystem/results/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mmarathe/Documents/GitHub/my_CATS/CATS-CaliforniaTestSystem/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64AEAD93-EB22-764B-BE37-49D5EABED810}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2283A2DF-4EDC-E542-B952-FEC563F25A97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3260" yWindow="2260" windowWidth="28040" windowHeight="17180" xr2:uid="{8EB89366-2FE9-9C44-A971-9D86756AE5B2}"/>
+    <workbookView xWindow="12540" yWindow="3340" windowWidth="28040" windowHeight="17180" activeTab="2" xr2:uid="{8EB89366-2FE9-9C44-A971-9D86756AE5B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="4" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="12">
   <si>
     <t>Shasta</t>
   </si>
@@ -66,6 +68,15 @@
   </si>
   <si>
     <t>Week of March 19 - 25, 2019</t>
+  </si>
+  <si>
+    <t>Selected generators assumed to have no cost in baseline case</t>
+  </si>
+  <si>
+    <t>All hydro generators assumed to have $1/MWh cost. In greedy case, selected generators have market offers</t>
+  </si>
+  <si>
+    <t>Note: The min and max hydro limit was taken from GODEEP</t>
   </si>
 </sst>
 </file>
@@ -437,7 +448,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDDF099E-D281-6D42-A7FA-6C5C6EE7A7EC}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -518,6 +529,197 @@
         <v>8</v>
       </c>
     </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64F9C666-6E6E-5742-91F5-0C933BAACB80}">
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="26.1640625" customWidth="1"/>
+    <col min="6" max="6" width="34" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>850939</v>
+      </c>
+      <c r="C2">
+        <v>919334</v>
+      </c>
+      <c r="E2">
+        <f>100*(C2-B2)/B2</f>
+        <v>8.037591413720607</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>220833</v>
+      </c>
+      <c r="C3">
+        <v>239263</v>
+      </c>
+      <c r="E3">
+        <f t="shared" ref="E3:E4" si="0">100*(C3-B3)/B3</f>
+        <v>8.345672974600717</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4">
+        <v>13400</v>
+      </c>
+      <c r="C4">
+        <v>15675</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="0"/>
+        <v>16.977611940298509</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5891D445-BFC7-2447-BFD3-346843CDAB27}">
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="26.1640625" customWidth="1"/>
+    <col min="6" max="6" width="34" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>850939</v>
+      </c>
+      <c r="C2">
+        <v>884737</v>
+      </c>
+      <c r="E2">
+        <f>100*(C2-B2)/B2</f>
+        <v>3.9718475707424385</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>220833</v>
+      </c>
+      <c r="C3">
+        <v>229606</v>
+      </c>
+      <c r="E3">
+        <f t="shared" ref="E3:E4" si="0">100*(C3-B3)/B3</f>
+        <v>3.9726852417890441</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4">
+        <v>13400</v>
+      </c>
+      <c r="C4">
+        <v>14338</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>